<commit_message>
feat: actualizar SKU_Cliente desde app de POs para P20321-15-11, P20321-15-12 y articulos recientes
</commit_message>
<xml_diff>
--- a/BD_SKUs_Autorizados.xlsx
+++ b/BD_SKUs_Autorizados.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1999" uniqueCount="1999">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2006" uniqueCount="2006">
   <si>
     <t>SKU</t>
   </si>
@@ -6011,6 +6011,27 @@
   </si>
   <si>
     <t>S/N</t>
+  </si>
+  <si>
+    <t>P20321-15-11</t>
+  </si>
+  <si>
+    <t>P20321-15-12</t>
+  </si>
+  <si>
+    <t>13-D-6195-01</t>
+  </si>
+  <si>
+    <t>13-D-6196-01</t>
+  </si>
+  <si>
+    <t>P20153S-04</t>
+  </si>
+  <si>
+    <t>P20321S-05</t>
+  </si>
+  <si>
+    <t>P20321S-06</t>
   </si>
 </sst>
 </file>
@@ -6342,7 +6363,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A1999"/>
+  <dimension ref="A1:A2006"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -16340,6 +16361,41 @@
         <v>1998</v>
       </c>
     </row>
+    <row r="2000" spans="1:1">
+      <c r="A2000" t="s">
+        <v>1999</v>
+      </c>
+    </row>
+    <row r="2001" spans="1:1">
+      <c r="A2001" t="s">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="2002" spans="1:1">
+      <c r="A2002" t="s">
+        <v>2001</v>
+      </c>
+    </row>
+    <row r="2003" spans="1:1">
+      <c r="A2003" t="s">
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="2004" spans="1:1">
+      <c r="A2004" t="s">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="2005" spans="1:1">
+      <c r="A2005" t="s">
+        <v>2004</v>
+      </c>
+    </row>
+    <row r="2006" spans="1:1">
+      <c r="A2006" t="s">
+        <v>2005</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: inyectar y dar de alta numeros de parte Proyecto TORONTO (TRTO/TRT0)
</commit_message>
<xml_diff>
--- a/BD_SKUs_Autorizados.xlsx
+++ b/BD_SKUs_Autorizados.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2006" uniqueCount="2006">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2030" uniqueCount="2030">
   <si>
     <t>SKU</t>
   </si>
@@ -6032,6 +6032,78 @@
   </si>
   <si>
     <t>P20321S-06</t>
+  </si>
+  <si>
+    <t>PP21139-092 TRTO</t>
+  </si>
+  <si>
+    <t>PP21139-092 TRT0</t>
+  </si>
+  <si>
+    <t>P9711-081 TRTO 2</t>
+  </si>
+  <si>
+    <t>P9711-081 TRT0 2</t>
+  </si>
+  <si>
+    <t>P7911-081 TRTO 1</t>
+  </si>
+  <si>
+    <t>P7911-081 TRT0 1</t>
+  </si>
+  <si>
+    <t>P9711-081 TRTO 1</t>
+  </si>
+  <si>
+    <t>P9711-081 TRT0 1</t>
+  </si>
+  <si>
+    <t>PP8655 TRTO-1</t>
+  </si>
+  <si>
+    <t>PP8655 TRT0-1</t>
+  </si>
+  <si>
+    <t>PP8655 TRTO</t>
+  </si>
+  <si>
+    <t>PP8655 TRT0</t>
+  </si>
+  <si>
+    <t>PP8655 TRTO1</t>
+  </si>
+  <si>
+    <t>PP8655 TRT01</t>
+  </si>
+  <si>
+    <t>PP8655-TRTO-1</t>
+  </si>
+  <si>
+    <t>PP8655-TRT0-1</t>
+  </si>
+  <si>
+    <t>P9711-081 TRTO</t>
+  </si>
+  <si>
+    <t>P9711-081 TRT0</t>
+  </si>
+  <si>
+    <t>PP21139-081 TRTO</t>
+  </si>
+  <si>
+    <t>PP21139-081 TRT0</t>
+  </si>
+  <si>
+    <t>11-C-9778-01 TRTO</t>
+  </si>
+  <si>
+    <t>11-C-9778-01 TRT0</t>
+  </si>
+  <si>
+    <t>PP21139-092</t>
+  </si>
+  <si>
+    <t>PP21139-081</t>
   </si>
 </sst>
 </file>
@@ -6363,7 +6435,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A2006"/>
+  <dimension ref="A1:A2030"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -16396,6 +16468,126 @@
         <v>2005</v>
       </c>
     </row>
+    <row r="2007" spans="1:1">
+      <c r="A2007" t="s">
+        <v>2006</v>
+      </c>
+    </row>
+    <row r="2008" spans="1:1">
+      <c r="A2008" t="s">
+        <v>2007</v>
+      </c>
+    </row>
+    <row r="2009" spans="1:1">
+      <c r="A2009" t="s">
+        <v>2008</v>
+      </c>
+    </row>
+    <row r="2010" spans="1:1">
+      <c r="A2010" t="s">
+        <v>2009</v>
+      </c>
+    </row>
+    <row r="2011" spans="1:1">
+      <c r="A2011" t="s">
+        <v>2010</v>
+      </c>
+    </row>
+    <row r="2012" spans="1:1">
+      <c r="A2012" t="s">
+        <v>2011</v>
+      </c>
+    </row>
+    <row r="2013" spans="1:1">
+      <c r="A2013" t="s">
+        <v>2012</v>
+      </c>
+    </row>
+    <row r="2014" spans="1:1">
+      <c r="A2014" t="s">
+        <v>2013</v>
+      </c>
+    </row>
+    <row r="2015" spans="1:1">
+      <c r="A2015" t="s">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="2016" spans="1:1">
+      <c r="A2016" t="s">
+        <v>2015</v>
+      </c>
+    </row>
+    <row r="2017" spans="1:1">
+      <c r="A2017" t="s">
+        <v>2016</v>
+      </c>
+    </row>
+    <row r="2018" spans="1:1">
+      <c r="A2018" t="s">
+        <v>2017</v>
+      </c>
+    </row>
+    <row r="2019" spans="1:1">
+      <c r="A2019" t="s">
+        <v>2018</v>
+      </c>
+    </row>
+    <row r="2020" spans="1:1">
+      <c r="A2020" t="s">
+        <v>2019</v>
+      </c>
+    </row>
+    <row r="2021" spans="1:1">
+      <c r="A2021" t="s">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="2022" spans="1:1">
+      <c r="A2022" t="s">
+        <v>2021</v>
+      </c>
+    </row>
+    <row r="2023" spans="1:1">
+      <c r="A2023" t="s">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="2024" spans="1:1">
+      <c r="A2024" t="s">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="2025" spans="1:1">
+      <c r="A2025" t="s">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2026" spans="1:1">
+      <c r="A2026" t="s">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="2027" spans="1:1">
+      <c r="A2027" t="s">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="2028" spans="1:1">
+      <c r="A2028" t="s">
+        <v>2027</v>
+      </c>
+    </row>
+    <row r="2029" spans="1:1">
+      <c r="A2029" t="s">
+        <v>2028</v>
+      </c>
+    </row>
+    <row r="2030" spans="1:1">
+      <c r="A2030" t="s">
+        <v>2029</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>